<commit_message>
docs(pre-audit): improve introduction, tools, and manual verification pages
</commit_message>
<xml_diff>
--- a/.storybook/public/documents/Checklist_pre-audit_CNAM_NOM_DU_PRODUIT.xlsx
+++ b/.storybook/public/documents/Checklist_pre-audit_CNAM_NOM_DU_PRODUIT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julien.Roche/code/cnam/design-system-v3/.storybook/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DB499A-CB48-E342-BBFA-03D4AE5734A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258AD8A1-76FD-5A4E-92B1-FAF7E6934166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{352E66E6-3C64-8D43-8BDA-4113AEA1A882}"/>
+    <workbookView xWindow="20240" yWindow="680" windowWidth="10000" windowHeight="17720" activeTab="2" xr2:uid="{352E66E6-3C64-8D43-8BDA-4113AEA1A882}"/>
   </bookViews>
   <sheets>
     <sheet name="Informations" sheetId="2" r:id="rId1"/>
@@ -52,22 +52,7 @@
     <t>2. Éléments visuels et déclenchements automatiques</t>
   </si>
   <si>
-    <t>3. Pertinence des liens et des boutons</t>
-  </si>
-  <si>
     <t>4. Formulaires</t>
-  </si>
-  <si>
-    <t>5. Tableaux accessibles</t>
-  </si>
-  <si>
-    <t>6. Langue de la page</t>
-  </si>
-  <si>
-    <t>7. Titre de la page</t>
-  </si>
-  <si>
-    <t>8. Accès aux contenus multimédia</t>
   </si>
   <si>
     <t>Conformité</t>
@@ -361,6 +346,21 @@
 7- Les contenus des intranets et des extranets publiés avant le 23 septembre 2019, jusqu’à ce que ces sites fassent l’objet d’une révision en profondeur ;
 8- Les contenus des sites internet et des applications mobiles qui ne sont ni nécessaires à l’accomplissement d’une démarche administrative active ni mis à jour ou modifiés après le 23 septembre 2019, notamment les archives.</t>
     </r>
+  </si>
+  <si>
+    <t>3. Pertinence des libellés et des textes alternatifs</t>
+  </si>
+  <si>
+    <t>5. Tableaux</t>
+  </si>
+  <si>
+    <t>6. Langue</t>
+  </si>
+  <si>
+    <t>7. Titre de la page et hiérarchie des titres</t>
+  </si>
+  <si>
+    <t>8. Contenus multimédia</t>
   </si>
 </sst>
 </file>
@@ -1462,7 +1462,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B1" s="28"/>
     </row>
@@ -1472,7 +1472,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="29" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B3" s="30"/>
     </row>
@@ -1482,51 +1482,51 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B7" s="5"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B8" s="5"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B9" s="5"/>
     </row>
     <row r="10" spans="1:2" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B10" s="5"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:2" ht="95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B12" s="5"/>
     </row>
@@ -1585,7 +1585,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B1" s="28"/>
     </row>
@@ -1595,7 +1595,7 @@
     </row>
     <row r="3" spans="1:4" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
@@ -1606,14 +1606,14 @@
     </row>
     <row r="5" spans="1:4" ht="271" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="32" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
     </row>
     <row r="7" spans="1:4" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D7" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1622,7 +1622,7 @@
     </row>
     <row r="9" spans="1:4" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="31" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B9" s="31"/>
       <c r="C9" s="31"/>
@@ -1636,7 +1636,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="18"/>
@@ -1650,91 +1650,91 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C14" s="22"/>
       <c r="D14" s="24"/>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="24"/>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
     </row>
     <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="24"/>
     </row>
     <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="24"/>
     </row>
     <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
     </row>
     <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="24"/>
     </row>
     <row r="21" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="23" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B22" s="23"/>
       <c r="C22" s="23"/>
@@ -1750,7 +1750,7 @@
     </row>
     <row r="23" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="23" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B23" s="23"/>
       <c r="C23" s="23"/>
@@ -1758,7 +1758,7 @@
     </row>
     <row r="24" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="23" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B24" s="23"/>
       <c r="C24" s="23"/>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="25" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="23" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -1829,7 +1829,7 @@
     </row>
     <row r="3" spans="1:3" ht="77" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="35" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -1841,32 +1841,32 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C5" s="34"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C6" s="34"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B7" s="34"/>
       <c r="C7" s="34"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B8" s="34"/>
       <c r="C8" s="34"/>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -1888,10 +1888,10 @@
         <v>0</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -1899,7 +1899,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C12" s="11"/>
     </row>
@@ -1908,61 +1908,61 @@
         <v>2</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C14" s="11"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C15" s="11"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C16" s="11"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C17" s="11"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C18" s="11"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C19" s="14"/>
     </row>
@@ -1973,7 +1973,7 @@
     </row>
     <row r="21" spans="1:3" ht="171" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="33"/>

</xml_diff>

<commit_message>
docs(pre-audit): improve introduction, tools, and manual verification pages (#1651)
</commit_message>
<xml_diff>
--- a/.storybook/public/documents/Checklist_pre-audit_CNAM_NOM_DU_PRODUIT.xlsx
+++ b/.storybook/public/documents/Checklist_pre-audit_CNAM_NOM_DU_PRODUIT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Julien.Roche/code/cnam/design-system-v3/.storybook/public/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DB499A-CB48-E342-BBFA-03D4AE5734A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258AD8A1-76FD-5A4E-92B1-FAF7E6934166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{352E66E6-3C64-8D43-8BDA-4113AEA1A882}"/>
+    <workbookView xWindow="20240" yWindow="680" windowWidth="10000" windowHeight="17720" activeTab="2" xr2:uid="{352E66E6-3C64-8D43-8BDA-4113AEA1A882}"/>
   </bookViews>
   <sheets>
     <sheet name="Informations" sheetId="2" r:id="rId1"/>
@@ -52,22 +52,7 @@
     <t>2. Éléments visuels et déclenchements automatiques</t>
   </si>
   <si>
-    <t>3. Pertinence des liens et des boutons</t>
-  </si>
-  <si>
     <t>4. Formulaires</t>
-  </si>
-  <si>
-    <t>5. Tableaux accessibles</t>
-  </si>
-  <si>
-    <t>6. Langue de la page</t>
-  </si>
-  <si>
-    <t>7. Titre de la page</t>
-  </si>
-  <si>
-    <t>8. Accès aux contenus multimédia</t>
   </si>
   <si>
     <t>Conformité</t>
@@ -361,6 +346,21 @@
 7- Les contenus des intranets et des extranets publiés avant le 23 septembre 2019, jusqu’à ce que ces sites fassent l’objet d’une révision en profondeur ;
 8- Les contenus des sites internet et des applications mobiles qui ne sont ni nécessaires à l’accomplissement d’une démarche administrative active ni mis à jour ou modifiés après le 23 septembre 2019, notamment les archives.</t>
     </r>
+  </si>
+  <si>
+    <t>3. Pertinence des libellés et des textes alternatifs</t>
+  </si>
+  <si>
+    <t>5. Tableaux</t>
+  </si>
+  <si>
+    <t>6. Langue</t>
+  </si>
+  <si>
+    <t>7. Titre de la page et hiérarchie des titres</t>
+  </si>
+  <si>
+    <t>8. Contenus multimédia</t>
   </si>
 </sst>
 </file>
@@ -1462,7 +1462,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B1" s="28"/>
     </row>
@@ -1472,7 +1472,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="29" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B3" s="30"/>
     </row>
@@ -1482,51 +1482,51 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B5" s="5"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B7" s="5"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B8" s="5"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B9" s="5"/>
     </row>
     <row r="10" spans="1:2" ht="87" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B10" s="5"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:2" ht="95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B12" s="5"/>
     </row>
@@ -1585,7 +1585,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B1" s="28"/>
     </row>
@@ -1595,7 +1595,7 @@
     </row>
     <row r="3" spans="1:4" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
@@ -1606,14 +1606,14 @@
     </row>
     <row r="5" spans="1:4" ht="271" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="32" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B5" s="32"/>
       <c r="C5" s="32"/>
     </row>
     <row r="7" spans="1:4" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D7" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1622,7 +1622,7 @@
     </row>
     <row r="9" spans="1:4" ht="115" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="31" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B9" s="31"/>
       <c r="C9" s="31"/>
@@ -1636,7 +1636,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="18"/>
@@ -1650,91 +1650,91 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C14" s="22"/>
       <c r="D14" s="24"/>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="24"/>
     </row>
     <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
     </row>
     <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" s="25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="24"/>
     </row>
     <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="24"/>
     </row>
     <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
     </row>
     <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="24"/>
     </row>
     <row r="21" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="23" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="23" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B22" s="23"/>
       <c r="C22" s="23"/>
@@ -1750,7 +1750,7 @@
     </row>
     <row r="23" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="23" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B23" s="23"/>
       <c r="C23" s="23"/>
@@ -1758,7 +1758,7 @@
     </row>
     <row r="24" spans="1:4" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="23" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B24" s="23"/>
       <c r="C24" s="23"/>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="25" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="23" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -1829,7 +1829,7 @@
     </row>
     <row r="3" spans="1:3" ht="77" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="35" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -1841,32 +1841,32 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C5" s="34"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C6" s="34"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B7" s="34"/>
       <c r="C7" s="34"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B8" s="34"/>
       <c r="C8" s="34"/>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -1888,10 +1888,10 @@
         <v>0</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -1899,7 +1899,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C12" s="11"/>
     </row>
@@ -1908,61 +1908,61 @@
         <v>2</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C13" s="11"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C14" s="11"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C15" s="11"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C16" s="11"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C17" s="11"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C18" s="11"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C19" s="14"/>
     </row>
@@ -1973,7 +1973,7 @@
     </row>
     <row r="21" spans="1:3" ht="171" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="33"/>

</xml_diff>